<commit_message>
Ad schedule spreadsheet: whole week (Mon as scheduled, Tue pack, Wed-Sun plan), workplan, totals per platform
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012br7gxAPU9SrRXphZmiNkC
</commit_message>
<xml_diff>
--- a/campaigns/AD-SCHEDULE.xlsx
+++ b/campaigns/AD-SCHEDULE.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workplan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule'!$A$3:$M$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule'!$A$3:$M$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -839,7 +839,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>IG + FB Story</t>
+          <t>Stories (Insta + Face)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1250,12 +1250,12 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Reel: bedtime story PART 2 (promised!)</t>
+          <t>Reel: bedtime story PART 2 (promised Mon)</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Claude makes (pack for tomorrow)</t>
+          <t>campaigns/2026-10-06/instagram-facebook/1-nico-story-part2.mp4</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>TikTok + YouTube Shorts</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Video: 30 minutes. Zero screens. (voice)</t>
+          <t>Video: bedtime story part 1</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>campaigns/nico/videos/screenfree-voice-music.mp4</t>
+          <t>campaigns/2026-10-06/tiktok/1-nico-story-part1.mp4</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -1345,27 +1345,27 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>YouTube Shorts</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Benny</t>
+          <t>Nico</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Video: can your 4-year-old read this? (voice)</t>
+          <t>Short: bedtime story part 1</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>campaigns/benny/videos/can-they-read-voice.mp4</t>
+          <t>campaigns/2026-10-06/youtube/1-nico-story-part1.mp4</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1400,37 +1400,33 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>YouTube Shorts</t>
+          <t>Stories (Insta + Face)</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Benny</t>
+          <t>Nico</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Short: same page 3 ways (voice)</t>
+          <t>Story with Link sticker</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>campaigns/benny/videos/yt-3-ways-voice.mp4</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
+          <t>(share the 19:00 Reel)</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr"/>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
@@ -1455,27 +1451,27 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Pinterest</t>
+          <t>IG + FB</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Nico</t>
+          <t>Benny</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Image pin: before/after</t>
+          <t>Reel: Can you find Bella?</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>campaigns/2026-10-05/pinterest/2-nico-pin-before-after.png</t>
+          <t>campaigns/2026-10-06/instagram-facebook/2-benny-find-bella.mp4</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -1485,7 +1481,7 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
+          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
@@ -1498,49 +1494,49 @@
       <c r="M19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>TikTok + YT + IG + FB</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Nico</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Carousel video: gift (voice)</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>campaigns/nico/videos/carousel-gift-voice.mp4</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Video: Can you find Bella?</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>campaigns/2026-10-06/tiktok/2-benny-find-bella.mp4</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>In that day's CAPTIONS.md</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
@@ -1550,50 +1546,50 @@
       </c>
       <c r="K20" s="5" t="inlineStr"/>
       <c r="L20" s="5" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>TikTok + YouTube Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>YouTube Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Benny</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Video (new)</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Claude makes</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Short: Can you find Bella?</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>campaigns/2026-10-06/youtube/2-yt-benny-find-bella.mp4</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>In that day's CAPTIONS.md</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
         </is>
@@ -1605,52 +1601,52 @@
       </c>
       <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="inlineStr"/>
-      <c r="M21" s="4" t="inlineStr"/>
+      <c r="M21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Pinterest</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Benny</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Nico</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Image pin: before/after</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>campaigns/2026-10-05/pinterest/3-benny-pin-before-after.png</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>campaigns/2026-10-06/pinterest/1-nico-pin-before-after.png</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>In that day's CAPTIONS.md</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -1660,50 +1656,46 @@
       </c>
       <c r="K22" s="5" t="inlineStr"/>
       <c r="L22" s="5" t="inlineStr"/>
-      <c r="M22" s="4" t="inlineStr"/>
+      <c r="M22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>TikTok + YT + IG + FB</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>IG + FB</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Nico</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Video: new coloring page (voice)</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Reel: bedtime story PART 3</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
@@ -1715,52 +1707,48 @@
       </c>
       <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="5" t="inlineStr"/>
-      <c r="M23" s="6" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>IG + FB + TikTok</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>Benny</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Photo carousel: gift</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>campaigns/benny/carousel-gift/</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>TikTok + YouTube Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Nico</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Video: bedtime story part 2</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>campaigns/nico/videos/bedtime-story-part2-voice-music.mp4</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -1770,50 +1758,46 @@
       </c>
       <c r="K24" s="5" t="inlineStr"/>
       <c r="L24" s="5" t="inlineStr"/>
-      <c r="M24" s="6" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>TikTok + YouTube Shorts</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>TikTok + YT + IG + FB</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Benny</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Video (new, real colors)</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
         </is>
@@ -1825,52 +1809,52 @@
       </c>
       <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="5" t="inlineStr"/>
-      <c r="M25" s="6" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Pinterest</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Nico</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Claude makes</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Image pin: before/after</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>campaigns/2026-10-05/pinterest/3-benny-pin-before-after.png</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>In that day's CAPTIONS.md</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -1880,50 +1864,46 @@
       </c>
       <c r="K26" s="5" t="inlineStr"/>
       <c r="L26" s="5" t="inlineStr"/>
-      <c r="M26" s="6" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>TikTok + YT + IG + FB</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Nico</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Video (new coloring page, voice)</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
@@ -1935,52 +1915,48 @@
       </c>
       <c r="K27" s="5" t="inlineStr"/>
       <c r="L27" s="5" t="inlineStr"/>
-      <c r="M27" s="4" t="inlineStr"/>
+      <c r="M27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>21:00</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>TikTok + YouTube Shorts</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>Nico</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>Claude makes</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>IG + FB + TikTok</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Photo carousel: gift</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>campaigns/benny/carousel-gift/</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -1990,52 +1966,48 @@
       </c>
       <c r="K28" s="5" t="inlineStr"/>
       <c r="L28" s="5" t="inlineStr"/>
-      <c r="M28" s="4" t="inlineStr"/>
+      <c r="M28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Pinterest</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Nico</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>TikTok + YT + IG + FB</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
+      <c r="H29" s="6" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -2045,27 +2017,27 @@
       </c>
       <c r="K29" s="5" t="inlineStr"/>
       <c r="L29" s="5" t="inlineStr"/>
-      <c r="M29" s="4" t="inlineStr"/>
+      <c r="M29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>TikTok + YT + IG + FB</t>
+          <t>Pinterest</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
@@ -2075,7 +2047,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Pin</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2083,11 +2055,7 @@
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
+      <c r="H30" s="6" t="inlineStr"/>
       <c r="I30" s="6" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
@@ -2103,47 +2071,43 @@
       <c r="M30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>IG + FB + TikTok</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>TikTok + YT + IG + FB</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>Nico</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>Photo carousel: story</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
@@ -2155,52 +2119,48 @@
       </c>
       <c r="K31" s="5" t="inlineStr"/>
       <c r="L31" s="5" t="inlineStr"/>
-      <c r="M31" s="6" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>TikTok + YouTube Shorts</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Benny</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>TikTok + YT + IG + FB</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Nico</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+      <c r="H32" s="4" t="inlineStr"/>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
@@ -2210,52 +2170,48 @@
       </c>
       <c r="K32" s="5" t="inlineStr"/>
       <c r="L32" s="5" t="inlineStr"/>
-      <c r="M32" s="6" t="inlineStr"/>
+      <c r="M32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Pinterest</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>Benny</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Nico</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+      <c r="H33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
@@ -2265,50 +2221,46 @@
       </c>
       <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="5" t="inlineStr"/>
-      <c r="M33" s="6" t="inlineStr"/>
+      <c r="M33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>TikTok + YT + IG + FB</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Nico</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr"/>
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
@@ -2320,52 +2272,48 @@
       </c>
       <c r="K34" s="5" t="inlineStr"/>
       <c r="L34" s="5" t="inlineStr"/>
-      <c r="M34" s="4" t="inlineStr"/>
+      <c r="M34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>TikTok + YouTube Shorts</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Benny</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>IG + FB + TikTok</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Nico</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Photo carousel: story</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+      <c r="H35" s="6" t="inlineStr"/>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
@@ -2375,52 +2323,48 @@
       </c>
       <c r="K35" s="5" t="inlineStr"/>
       <c r="L35" s="5" t="inlineStr"/>
-      <c r="M35" s="4" t="inlineStr"/>
+      <c r="M35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Pinterest</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Nico</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>TikTok + YT + IG + FB</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>Claude makes</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
+      <c r="H36" s="6" t="inlineStr"/>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
@@ -2430,46 +2374,50 @@
       </c>
       <c r="K36" s="5" t="inlineStr"/>
       <c r="L36" s="5" t="inlineStr"/>
-      <c r="M36" s="4" t="inlineStr"/>
+      <c r="M36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Sunday check</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>KDP sales + best posts -&gt; tell Claude</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>In that day's CAPTIONS.md</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Claude makes</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr"/>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+        </is>
+      </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2477,12 +2425,208 @@
       </c>
       <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="5" t="inlineStr"/>
-      <c r="M37" s="4" t="inlineStr"/>
+      <c r="M37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>TikTok + YT + IG + FB</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Nico</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Claude makes</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr"/>
+      <c r="L38" s="5" t="inlineStr"/>
+      <c r="M38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>TikTok + YT + IG + FB</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Claude makes</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVSLXK7</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr"/>
+      <c r="L39" s="5" t="inlineStr"/>
+      <c r="M39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Nico</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Claude makes</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0HLVTTK7T</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr"/>
+      <c r="L40" s="5" t="inlineStr"/>
+      <c r="M40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Sunday check</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>KDP sales + best posts: tell Claude</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr"/>
+      <c r="L41" s="5" t="inlineStr"/>
+      <c r="M41" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M37"/>
+  <autoFilter ref="A3:M41"/>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Planned,To do,Scheduled,Posted,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2547,15 +2691,15 @@
         </is>
       </c>
       <c r="B3" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*TikTok*",Schedule!$J$4:$J$37,"Planned")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*TikTok*",Schedule!$J$4:$J$41,"Planned")</f>
         <v/>
       </c>
       <c r="C3" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*TikTok*",Schedule!$J$4:$J$37,"Scheduled")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*TikTok*",Schedule!$J$4:$J$41,"Scheduled")</f>
         <v/>
       </c>
       <c r="D3" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*TikTok*",Schedule!$J$4:$J$37,"Posted")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*TikTok*",Schedule!$J$4:$J$41,"Posted")</f>
         <v/>
       </c>
       <c r="E3" s="9">
@@ -2570,15 +2714,15 @@
         </is>
       </c>
       <c r="B4" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*YouTube*",Schedule!$J$4:$J$37,"Planned")+COUNTIFS(Schedule!$D$4:$D$37,"*YT*",Schedule!$J$4:$J$37,"Planned")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*YouTube*",Schedule!$J$4:$J$41,"Planned")+COUNTIFS(Schedule!$D$4:$D$41,"*YT*",Schedule!$J$4:$J$41,"Planned")</f>
         <v/>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*YouTube*",Schedule!$J$4:$J$37,"Scheduled")+COUNTIFS(Schedule!$D$4:$D$37,"*YT*",Schedule!$J$4:$J$37,"Scheduled")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*YouTube*",Schedule!$J$4:$J$41,"Scheduled")+COUNTIFS(Schedule!$D$4:$D$41,"*YT*",Schedule!$J$4:$J$41,"Scheduled")</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*YouTube*",Schedule!$J$4:$J$37,"Posted")+COUNTIFS(Schedule!$D$4:$D$37,"*YT*",Schedule!$J$4:$J$37,"Posted")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*YouTube*",Schedule!$J$4:$J$41,"Posted")+COUNTIFS(Schedule!$D$4:$D$41,"*YT*",Schedule!$J$4:$J$41,"Posted")</f>
         <v/>
       </c>
       <c r="E4" s="9">
@@ -2593,15 +2737,15 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Instagram*",Schedule!$J$4:$J$37,"Planned")+COUNTIFS(Schedule!$D$4:$D$37,"*IG*",Schedule!$J$4:$J$37,"Planned")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Instagram*",Schedule!$J$4:$J$41,"Planned")+COUNTIFS(Schedule!$D$4:$D$41,"*IG*",Schedule!$J$4:$J$41,"Planned")</f>
         <v/>
       </c>
       <c r="C5" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Instagram*",Schedule!$J$4:$J$37,"Scheduled")+COUNTIFS(Schedule!$D$4:$D$37,"*IG*",Schedule!$J$4:$J$37,"Scheduled")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Instagram*",Schedule!$J$4:$J$41,"Scheduled")+COUNTIFS(Schedule!$D$4:$D$41,"*IG*",Schedule!$J$4:$J$41,"Scheduled")</f>
         <v/>
       </c>
       <c r="D5" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Instagram*",Schedule!$J$4:$J$37,"Posted")+COUNTIFS(Schedule!$D$4:$D$37,"*IG*",Schedule!$J$4:$J$37,"Posted")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Instagram*",Schedule!$J$4:$J$41,"Posted")+COUNTIFS(Schedule!$D$4:$D$41,"*IG*",Schedule!$J$4:$J$41,"Posted")</f>
         <v/>
       </c>
       <c r="E5" s="9">
@@ -2616,15 +2760,15 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Facebook*",Schedule!$J$4:$J$37,"Planned")+COUNTIFS(Schedule!$D$4:$D$37,"*FB*",Schedule!$J$4:$J$37,"Planned")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Facebook*",Schedule!$J$4:$J$41,"Planned")+COUNTIFS(Schedule!$D$4:$D$41,"*FB*",Schedule!$J$4:$J$41,"Planned")</f>
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Facebook*",Schedule!$J$4:$J$37,"Scheduled")+COUNTIFS(Schedule!$D$4:$D$37,"*FB*",Schedule!$J$4:$J$37,"Scheduled")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Facebook*",Schedule!$J$4:$J$41,"Scheduled")+COUNTIFS(Schedule!$D$4:$D$41,"*FB*",Schedule!$J$4:$J$41,"Scheduled")</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Facebook*",Schedule!$J$4:$J$37,"Posted")+COUNTIFS(Schedule!$D$4:$D$37,"*FB*",Schedule!$J$4:$J$37,"Posted")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Facebook*",Schedule!$J$4:$J$41,"Posted")+COUNTIFS(Schedule!$D$4:$D$41,"*FB*",Schedule!$J$4:$J$41,"Posted")</f>
         <v/>
       </c>
       <c r="E6" s="9">
@@ -2639,15 +2783,15 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Pinterest*",Schedule!$J$4:$J$37,"Planned")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Pinterest*",Schedule!$J$4:$J$41,"Planned")</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Pinterest*",Schedule!$J$4:$J$37,"Scheduled")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Pinterest*",Schedule!$J$4:$J$41,"Scheduled")</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>COUNTIFS(Schedule!$D$4:$D$37,"*Pinterest*",Schedule!$J$4:$J$37,"Posted")</f>
+        <f>COUNTIFS(Schedule!$D$4:$D$41,"*Pinterest*",Schedule!$J$4:$J$41,"Posted")</f>
         <v/>
       </c>
       <c r="E7" s="9">
@@ -2779,7 +2923,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>1 Reel (19:00)</t>
+          <t>2 Reels, one per book (19:00 + 21:00)</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -2806,7 +2950,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>1 Reel (same as IG)</t>
+          <t>2 Reels (same as IG)</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">

</xml_diff>